<commit_message>
week 2 betting odds
</commit_message>
<xml_diff>
--- a/data/leagues/BP- Loudoun 2025 2026.xlsx
+++ b/data/leagues/BP- Loudoun 2025 2026.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="116">
   <si>
     <t>Bears, Jags, Foxes, Oh My!</t>
   </si>
@@ -250,13 +250,13 @@
     <t>10.5-3.3-0.1</t>
   </si>
   <si>
-    <t>9.3-4.7</t>
-  </si>
-  <si>
-    <t>9.3-4.6-0.1</t>
-  </si>
-  <si>
-    <t>8.7-5.1-0.2</t>
+    <t>9.4-4.5-0.1</t>
+  </si>
+  <si>
+    <t>9.2-4.7-0.1</t>
+  </si>
+  <si>
+    <t>8.7-5.2-0.2</t>
   </si>
   <si>
     <t>7.7-6.2-0.1</t>
@@ -265,25 +265,28 @@
     <t>7.1-6.7-0.1</t>
   </si>
   <si>
-    <t>6.8-7.1-0.1</t>
-  </si>
-  <si>
-    <t>5.7-8.2-0.1</t>
-  </si>
-  <si>
-    <t>5.1-8.8-0.1</t>
-  </si>
-  <si>
-    <t>4.9-9.0-0.1</t>
+    <t>6.8-7.0-0.1</t>
+  </si>
+  <si>
+    <t>5.8-8.1-0.1</t>
+  </si>
+  <si>
+    <t>5.0-8.9-0.1</t>
+  </si>
+  <si>
+    <t>4.8-9.1-0.1</t>
   </si>
   <si>
     <t>3.9-9.9-0.1</t>
   </si>
   <si>
+    <t>3.4-10.5-0.1</t>
+  </si>
+  <si>
     <t>3.6-10.3-0.1</t>
   </si>
   <si>
-    <t>3.3-10.6-0.1</t>
+    <t>12-2</t>
   </si>
   <si>
     <t>11-3</t>
@@ -292,13 +295,13 @@
     <t>9-5</t>
   </si>
   <si>
-    <t>10-4</t>
-  </si>
-  <si>
     <t>8-6</t>
   </si>
   <si>
     <t>7-7</t>
+  </si>
+  <si>
+    <t>6-8</t>
   </si>
   <si>
     <t>5-9</t>
@@ -1442,25 +1445,25 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="B1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2085,28 +2088,28 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <v>52.5</v>
+        <v>51.7</v>
       </c>
       <c r="C2">
-        <v>24.8</v>
+        <v>23</v>
       </c>
       <c r="D2">
-        <v>11.7</v>
+        <v>13.9</v>
       </c>
       <c r="E2">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="F2">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="G2">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="H2">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -2127,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>99.8</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -2138,28 +2141,28 @@
         <v>22.3</v>
       </c>
       <c r="C3">
-        <v>33.5</v>
+        <v>33.3</v>
       </c>
       <c r="D3">
-        <v>21.6</v>
+        <v>20.8</v>
       </c>
       <c r="E3">
-        <v>10.9</v>
+        <v>11.7</v>
       </c>
       <c r="F3">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="G3">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="H3">
-        <v>1.5</v>
+        <v>0.9</v>
       </c>
       <c r="I3">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="J3">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -2177,7 +2180,7 @@
         <v>0</v>
       </c>
       <c r="P3">
-        <v>98</v>
+        <v>98.2</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -2185,43 +2188,43 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>11.5</v>
+        <v>12.9</v>
       </c>
       <c r="C4">
-        <v>15.6</v>
+        <v>17.7</v>
       </c>
       <c r="D4">
-        <v>19.4</v>
+        <v>18.3</v>
       </c>
       <c r="E4">
-        <v>16.4</v>
+        <v>15.9</v>
       </c>
       <c r="F4">
-        <v>13.8</v>
+        <v>12.6</v>
       </c>
       <c r="G4">
-        <v>10</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H4">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="I4">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="J4">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="K4">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="L4">
         <v>0.5</v>
       </c>
       <c r="M4">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -2235,49 +2238,49 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>9.4</v>
+        <v>7.7</v>
       </c>
       <c r="C5">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="D5">
-        <v>19.2</v>
+        <v>18.3</v>
       </c>
       <c r="E5">
-        <v>20.2</v>
+        <v>18.9</v>
       </c>
       <c r="F5">
-        <v>13.6</v>
+        <v>14.5</v>
       </c>
       <c r="G5">
-        <v>10</v>
+        <v>10.7</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I5">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="J5">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="K5">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="L5">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="N5">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>85.7</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="6" spans="1:16">
@@ -2288,46 +2291,46 @@
         <v>1.7</v>
       </c>
       <c r="C6">
-        <v>6.8</v>
+        <v>6</v>
       </c>
       <c r="D6">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="E6">
-        <v>21.3</v>
+        <v>22.5</v>
       </c>
       <c r="F6">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
       <c r="G6">
-        <v>17.7</v>
+        <v>16</v>
       </c>
       <c r="H6">
-        <v>10.1</v>
+        <v>8.4</v>
       </c>
       <c r="I6">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="L6">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
         <v>0.1</v>
       </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>82.7</v>
+        <v>82.3</v>
       </c>
     </row>
     <row r="7" spans="1:16">
@@ -2335,49 +2338,49 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2.1</v>
+        <v>2.8</v>
       </c>
       <c r="C7">
-        <v>3.2</v>
+        <v>4.9</v>
       </c>
       <c r="D7">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="E7">
-        <v>10.6</v>
+        <v>10.2</v>
       </c>
       <c r="F7">
-        <v>15.4</v>
+        <v>16.5</v>
       </c>
       <c r="G7">
-        <v>18.1</v>
+        <v>18.5</v>
       </c>
       <c r="H7">
-        <v>15.5</v>
+        <v>13.6</v>
       </c>
       <c r="I7">
-        <v>10.8</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J7">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="K7">
-        <v>4.4</v>
+        <v>4.9</v>
       </c>
       <c r="L7">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="M7">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="N7">
         <v>0.7</v>
       </c>
       <c r="O7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="P7">
-        <v>56.6</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:16">
@@ -2385,40 +2388,40 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="C8">
-        <v>2.1</v>
+        <v>1</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="E8">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="F8">
-        <v>11</v>
+        <v>10.5</v>
       </c>
       <c r="G8">
-        <v>14.1</v>
+        <v>16.3</v>
       </c>
       <c r="H8">
-        <v>18.5</v>
+        <v>17.1</v>
       </c>
       <c r="I8">
-        <v>15.4</v>
+        <v>17.2</v>
       </c>
       <c r="J8">
-        <v>11.6</v>
+        <v>10.8</v>
       </c>
       <c r="K8">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="L8">
-        <v>4.7</v>
+        <v>5.3</v>
       </c>
       <c r="M8">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="N8">
         <v>1</v>
@@ -2427,7 +2430,7 @@
         <v>0.7</v>
       </c>
       <c r="P8">
-        <v>38.7</v>
+        <v>39.9</v>
       </c>
     </row>
     <row r="9" spans="1:16">
@@ -2438,46 +2441,46 @@
         <v>0.1</v>
       </c>
       <c r="C9">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D9">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="E9">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="F9">
         <v>7.7</v>
       </c>
       <c r="G9">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="H9">
-        <v>15.1</v>
+        <v>18.4</v>
       </c>
       <c r="I9">
-        <v>22.5</v>
+        <v>21.1</v>
       </c>
       <c r="J9">
-        <v>16.5</v>
+        <v>16</v>
       </c>
       <c r="K9">
-        <v>9.800000000000001</v>
+        <v>10.6</v>
       </c>
       <c r="L9">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="M9">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="N9">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O9">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="P9">
-        <v>26.9</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="10" spans="1:16">
@@ -2485,49 +2488,49 @@
         <v>4</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="C10">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E10">
-        <v>1.5</v>
+        <v>1.9</v>
       </c>
       <c r="F10">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="G10">
-        <v>6.8</v>
+        <v>7.9</v>
       </c>
       <c r="H10">
-        <v>12.7</v>
+        <v>11</v>
       </c>
       <c r="I10">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="J10">
-        <v>14.8</v>
+        <v>17</v>
       </c>
       <c r="K10">
-        <v>15.2</v>
+        <v>14.6</v>
       </c>
       <c r="L10">
-        <v>12.6</v>
+        <v>11.1</v>
       </c>
       <c r="M10">
-        <v>8.1</v>
+        <v>7.4</v>
       </c>
       <c r="N10">
-        <v>5.7</v>
+        <v>7.2</v>
       </c>
       <c r="O10">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="P10">
-        <v>13.3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:16">
@@ -2544,40 +2547,40 @@
         <v>0.3</v>
       </c>
       <c r="E11">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="F11">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="G11">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="H11">
-        <v>5.3</v>
+        <v>6.3</v>
       </c>
       <c r="I11">
-        <v>9.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J11">
-        <v>13.6</v>
+        <v>11.8</v>
       </c>
       <c r="K11">
-        <v>15.6</v>
+        <v>14.3</v>
       </c>
       <c r="L11">
-        <v>16.2</v>
+        <v>17.1</v>
       </c>
       <c r="M11">
-        <v>15.1</v>
+        <v>15</v>
       </c>
       <c r="N11">
-        <v>12</v>
+        <v>12.1</v>
       </c>
       <c r="O11">
-        <v>7.8</v>
+        <v>10.2</v>
       </c>
       <c r="P11">
-        <v>5.2</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -2591,43 +2594,43 @@
         <v>0</v>
       </c>
       <c r="D12">
+        <v>0.1</v>
+      </c>
+      <c r="E12">
         <v>0.2</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>0.5</v>
       </c>
-      <c r="F12">
-        <v>1.2</v>
-      </c>
       <c r="G12">
-        <v>3</v>
+        <v>1.6</v>
       </c>
       <c r="H12">
-        <v>4.8</v>
+        <v>7.1</v>
       </c>
       <c r="I12">
-        <v>10.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12">
-        <v>16.7</v>
+        <v>13.9</v>
       </c>
       <c r="K12">
-        <v>17.9</v>
+        <v>17.7</v>
       </c>
       <c r="L12">
-        <v>15.1</v>
+        <v>17.1</v>
       </c>
       <c r="M12">
-        <v>13.5</v>
+        <v>14.1</v>
       </c>
       <c r="N12">
-        <v>10.2</v>
+        <v>11.6</v>
       </c>
       <c r="O12">
-        <v>6.8</v>
+        <v>7.3</v>
       </c>
       <c r="P12">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="13" spans="1:16">
@@ -2644,45 +2647,45 @@
         <v>0</v>
       </c>
       <c r="E13">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F13">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="G13">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="H13">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="I13">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="J13">
-        <v>5.2</v>
+        <v>8</v>
       </c>
       <c r="K13">
-        <v>12.5</v>
+        <v>11.8</v>
       </c>
       <c r="L13">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="M13">
-        <v>19.4</v>
+        <v>18</v>
       </c>
       <c r="N13">
-        <v>21.4</v>
+        <v>19.5</v>
       </c>
       <c r="O13">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
       <c r="P13">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -2697,42 +2700,42 @@
         <v>0</v>
       </c>
       <c r="F14">
+        <v>0.1</v>
+      </c>
+      <c r="G14">
+        <v>0.1</v>
+      </c>
+      <c r="H14">
+        <v>0.7</v>
+      </c>
+      <c r="I14">
+        <v>1.8</v>
+      </c>
+      <c r="J14">
+        <v>2.9</v>
+      </c>
+      <c r="K14">
+        <v>7.2</v>
+      </c>
+      <c r="L14">
+        <v>7.4</v>
+      </c>
+      <c r="M14">
+        <v>19.3</v>
+      </c>
+      <c r="N14">
+        <v>22.6</v>
+      </c>
+      <c r="O14">
+        <v>37.9</v>
+      </c>
+      <c r="P14">
         <v>0.2</v>
-      </c>
-      <c r="G14">
-        <v>0.3</v>
-      </c>
-      <c r="H14">
-        <v>0.9</v>
-      </c>
-      <c r="I14">
-        <v>1.7</v>
-      </c>
-      <c r="J14">
-        <v>4.8</v>
-      </c>
-      <c r="K14">
-        <v>10.1</v>
-      </c>
-      <c r="L14">
-        <v>15</v>
-      </c>
-      <c r="M14">
-        <v>22.1</v>
-      </c>
-      <c r="N14">
-        <v>25.4</v>
-      </c>
-      <c r="O14">
-        <v>19.5</v>
-      </c>
-      <c r="P14">
-        <v>0.5</v>
       </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2744,37 +2747,37 @@
         <v>0</v>
       </c>
       <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
         <v>0.1</v>
       </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
       <c r="H15">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="I15">
-        <v>1.8</v>
+        <v>2.3</v>
       </c>
       <c r="J15">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="K15">
-        <v>5.2</v>
+        <v>10.1</v>
       </c>
       <c r="L15">
-        <v>9.9</v>
+        <v>15.4</v>
       </c>
       <c r="M15">
-        <v>13.9</v>
+        <v>21.1</v>
       </c>
       <c r="N15">
-        <v>22.6</v>
+        <v>24.3</v>
       </c>
       <c r="O15">
-        <v>42.5</v>
+        <v>22</v>
       </c>
       <c r="P15">
         <v>0.1</v>
@@ -2806,13 +2809,13 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <v>95.5</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="C2">
-        <v>99.59999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2820,13 +2823,13 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>84.89999999999999</v>
+        <v>82.69999999999999</v>
       </c>
       <c r="C3">
-        <v>99.09999999999999</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="D3">
-        <v>98</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2834,13 +2837,13 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>18.8</v>
+        <v>19.8</v>
       </c>
       <c r="C4">
-        <v>82.39999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="D4">
-        <v>87</v>
+        <v>85.39999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2851,10 +2854,10 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C5">
-        <v>87.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="D5">
-        <v>86.90000000000001</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2862,13 +2865,13 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>70.89999999999999</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="C6">
-        <v>79.7</v>
+        <v>79.60000000000001</v>
       </c>
       <c r="D6">
-        <v>81</v>
+        <v>81.89999999999999</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2879,10 +2882,10 @@
         <v>0.7000000000000001</v>
       </c>
       <c r="C7">
-        <v>54.90000000000001</v>
+        <v>56.39999999999999</v>
       </c>
       <c r="D7">
-        <v>54.8</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2890,13 +2893,13 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>83.89999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="C8">
-        <v>38</v>
+        <v>40.6</v>
       </c>
       <c r="D8">
-        <v>39.3</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2904,13 +2907,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>35.09999999999999</v>
+        <v>35.5</v>
       </c>
       <c r="C9">
-        <v>34.2</v>
+        <v>32.8</v>
       </c>
       <c r="D9">
-        <v>28.9</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2918,13 +2921,13 @@
         <v>4</v>
       </c>
       <c r="B10">
-        <v>53</v>
+        <v>53.2</v>
       </c>
       <c r="C10">
-        <v>13.7</v>
+        <v>11.6</v>
       </c>
       <c r="D10">
-        <v>12.8</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2932,13 +2935,13 @@
         <v>7</v>
       </c>
       <c r="B11">
-        <v>19.8</v>
+        <v>20.5</v>
       </c>
       <c r="C11">
-        <v>5.800000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="D11">
-        <v>6.600000000000001</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2946,13 +2949,13 @@
         <v>0</v>
       </c>
       <c r="B12">
-        <v>21.2</v>
+        <v>19.7</v>
       </c>
       <c r="C12">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="D12">
-        <v>3.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2960,41 +2963,41 @@
         <v>6</v>
       </c>
       <c r="B13">
-        <v>5.800000000000001</v>
+        <v>5.3</v>
       </c>
       <c r="C13">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="D13">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B14">
-        <v>7.3</v>
+        <v>3.3</v>
       </c>
       <c r="C14">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D14">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15">
-        <v>3.2</v>
+        <v>7.8</v>
       </c>
       <c r="C15">
+        <v>0.8999999999999999</v>
+      </c>
+      <c r="D15">
         <v>0.3</v>
-      </c>
-      <c r="D15">
-        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -3495,7 +3498,7 @@
         <v>241.4</v>
       </c>
       <c r="F2">
-        <v>99.8</v>
+        <v>99.5</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3524,7 +3527,7 @@
         <v>232.68</v>
       </c>
       <c r="F3">
-        <v>98</v>
+        <v>98.2</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -3533,7 +3536,7 @@
         <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -3562,7 +3565,7 @@
         <v>75</v>
       </c>
       <c r="I4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -3582,7 +3585,7 @@
         <v>221.58</v>
       </c>
       <c r="F5">
-        <v>85.7</v>
+        <v>83.3</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -3611,7 +3614,7 @@
         <v>220.44</v>
       </c>
       <c r="F6">
-        <v>82.69999999999999</v>
+        <v>82.3</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -3620,7 +3623,7 @@
         <v>77</v>
       </c>
       <c r="I6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -3640,10 +3643,10 @@
         <v>219.36</v>
       </c>
       <c r="F7">
-        <v>56.59999999999999</v>
+        <v>60</v>
       </c>
       <c r="G7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H7" t="s">
         <v>78</v>
@@ -3669,7 +3672,7 @@
         <v>204.94</v>
       </c>
       <c r="F8">
-        <v>38.7</v>
+        <v>39.90000000000001</v>
       </c>
       <c r="G8">
         <v>0.7000000000000001</v>
@@ -3698,10 +3701,10 @@
         <v>195.66</v>
       </c>
       <c r="F9">
-        <v>26.9</v>
+        <v>26.4</v>
       </c>
       <c r="G9">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="s">
         <v>80</v>
@@ -3727,10 +3730,10 @@
         <v>194.78</v>
       </c>
       <c r="F10">
-        <v>13.3</v>
+        <v>15</v>
       </c>
       <c r="G10">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="H10" t="s">
         <v>81</v>
@@ -3756,16 +3759,16 @@
         <v>168.7</v>
       </c>
       <c r="F11">
-        <v>5.2</v>
+        <v>4.9</v>
       </c>
       <c r="G11">
-        <v>7.8</v>
+        <v>10.2</v>
       </c>
       <c r="H11" t="s">
         <v>82</v>
       </c>
       <c r="I11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -3785,16 +3788,16 @@
         <v>186.96</v>
       </c>
       <c r="F12">
-        <v>4.9</v>
+        <v>2.4</v>
       </c>
       <c r="G12">
-        <v>6.800000000000001</v>
+        <v>7.3</v>
       </c>
       <c r="H12" t="s">
         <v>83</v>
       </c>
       <c r="I12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -3814,21 +3817,21 @@
         <v>175.84</v>
       </c>
       <c r="F13">
-        <v>0.8999999999999999</v>
+        <v>1.1</v>
       </c>
       <c r="G13">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
       <c r="H13" t="s">
         <v>84</v>
       </c>
       <c r="I13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B14" t="s">
         <v>72</v>
@@ -3837,27 +3840,27 @@
         <v>0</v>
       </c>
       <c r="D14">
-        <v>87.97999999999999</v>
+        <v>78.27</v>
       </c>
       <c r="E14">
-        <v>175.96</v>
+        <v>156.54</v>
       </c>
       <c r="F14">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="G14">
-        <v>19.5</v>
+        <v>37.9</v>
       </c>
       <c r="H14" t="s">
         <v>85</v>
       </c>
       <c r="I14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>72</v>
@@ -3866,22 +3869,22 @@
         <v>0</v>
       </c>
       <c r="D15">
-        <v>78.27</v>
+        <v>87.97999999999999</v>
       </c>
       <c r="E15">
-        <v>156.54</v>
+        <v>175.96</v>
       </c>
       <c r="F15">
         <v>0.1</v>
       </c>
       <c r="G15">
-        <v>42.5</v>
+        <v>22</v>
       </c>
       <c r="H15" t="s">
         <v>86</v>
       </c>
       <c r="I15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3899,16 +3902,16 @@
         <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3928,7 +3931,7 @@
         <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3948,7 +3951,7 @@
         <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -3968,7 +3971,7 @@
         <v>15</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3988,7 +3991,7 @@
         <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -4008,7 +4011,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -4028,7 +4031,7 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -4048,7 +4051,7 @@
         <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -4068,7 +4071,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4088,7 +4091,7 @@
         <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -4108,7 +4111,7 @@
         <v>15</v>
       </c>
       <c r="F11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -4128,7 +4131,7 @@
         <v>16</v>
       </c>
       <c r="F12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -4148,7 +4151,7 @@
         <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -4168,7 +4171,7 @@
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -4188,7 +4191,7 @@
         <v>14</v>
       </c>
       <c r="F15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -4203,13 +4206,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -4223,7 +4226,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4237,7 +4240,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -4251,7 +4254,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -4265,7 +4268,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -4279,7 +4282,7 @@
         <v>3</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -4293,7 +4296,7 @@
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -4307,7 +4310,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -4321,7 +4324,7 @@
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -4335,7 +4338,7 @@
         <v>-2</v>
       </c>
       <c r="D10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -4349,7 +4352,7 @@
         <v>-2</v>
       </c>
       <c r="D11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -4363,7 +4366,7 @@
         <v>-3</v>
       </c>
       <c r="D12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -4377,7 +4380,7 @@
         <v>-4</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -4391,7 +4394,7 @@
         <v>-5</v>
       </c>
       <c r="D14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -4405,7 +4408,7 @@
         <v>-15</v>
       </c>
       <c r="D15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>